<commit_message>
fix: break skeleton fall-apart/recombine conservation loop
Add monster.big_skeleton_reborn as a reserve variant without fall_apart.
Recombine skills now shuffle the reborn card instead of the native big
skeleton, preventing the 1-big-skeleton <-> 2-fragments infinite cycle.

Also exclude IsReserve cards from ShuffleRandomContent candidate pools,
update Luban/streaming data and content visual entries, and extend
RecombineDedup regression tests with a no-fall-apart kill case.

Co-authored-by: Tang Jin <tja688@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Assets/Tools/Luban/Datas/content_visual.xlsx
+++ b/Assets/Tools/Luban/Datas/content_visual.xlsx
@@ -1,34 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TbContentVisual" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TbContentVisual" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <name val="宋体"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -56,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -419,16 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D191"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="37.44140625" customWidth="1" min="2" max="2"/>
-    <col width="11.21875" customWidth="1" min="3" max="3"/>
-    <col width="172.109375" customWidth="1" min="4" max="4"/>
-    <col width="24.21875" customWidth="1" min="5" max="5"/>
-    <col width="11.109375" customWidth="1" min="6" max="6"/>
-    <col width="9.77734375" customWidth="1" min="7" max="7"/>
-  </cols>
+  <dimension ref="A1:D192"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -475,6 +461,7 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>avatar.default</t>
@@ -492,6 +479,7 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr"/>
       <c r="B4" t="inlineStr">
         <is>
           <t>help.armor_breaking_hammer</t>
@@ -509,6 +497,7 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr"/>
       <c r="B5" t="inlineStr">
         <is>
           <t>help.bear_trap</t>
@@ -526,6 +515,7 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>help.blood_conversion</t>
@@ -543,6 +533,7 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>help.blue_chest_card</t>
@@ -560,6 +551,7 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr"/>
       <c r="B8" t="inlineStr">
         <is>
           <t>help.bomb</t>
@@ -577,6 +569,7 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>help.brutality_card</t>
@@ -594,6 +587,7 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr">
         <is>
           <t>help.common_chest_card</t>
@@ -611,6 +605,7 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>help.doubling_tower</t>
@@ -628,6 +623,7 @@
       </c>
     </row>
     <row r="12">
+      <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr">
         <is>
           <t>help.fireball</t>
@@ -645,6 +641,7 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr">
         <is>
           <t>help.flame</t>
@@ -662,6 +659,7 @@
       </c>
     </row>
     <row r="14">
+      <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr">
         <is>
           <t>help.food_card</t>
@@ -679,6 +677,7 @@
       </c>
     </row>
     <row r="15">
+      <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr">
         <is>
           <t>help.gold_card</t>
@@ -696,6 +695,7 @@
       </c>
     </row>
     <row r="16">
+      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>help.golden_chest_card</t>
@@ -713,6 +713,7 @@
       </c>
     </row>
     <row r="17">
+      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>help.healing_potion</t>
@@ -730,6 +731,7 @@
       </c>
     </row>
     <row r="18">
+      <c r="A18" t="inlineStr"/>
       <c r="B18" t="inlineStr">
         <is>
           <t>help.healing_spring</t>
@@ -747,6 +749,7 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr"/>
       <c r="B19" t="inlineStr">
         <is>
           <t>help.impact_tutorial</t>
@@ -764,6 +767,7 @@
       </c>
     </row>
     <row r="20">
+      <c r="A20" t="inlineStr"/>
       <c r="B20" t="inlineStr">
         <is>
           <t>help.kidnapping</t>
@@ -781,6 +785,7 @@
       </c>
     </row>
     <row r="21">
+      <c r="A21" t="inlineStr"/>
       <c r="B21" t="inlineStr">
         <is>
           <t>help.rolling_stone</t>
@@ -798,6 +803,7 @@
       </c>
     </row>
     <row r="22">
+      <c r="A22" t="inlineStr"/>
       <c r="B22" t="inlineStr">
         <is>
           <t>help.rotation_wheel</t>
@@ -815,6 +821,7 @@
       </c>
     </row>
     <row r="23">
+      <c r="A23" t="inlineStr"/>
       <c r="B23" t="inlineStr">
         <is>
           <t>help.shield_bash_tutorial</t>
@@ -832,6 +839,7 @@
       </c>
     </row>
     <row r="24">
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr">
         <is>
           <t>help.stat_boost_card</t>
@@ -849,6 +857,7 @@
       </c>
     </row>
     <row r="25">
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr">
         <is>
           <t>help.sturdy_shield</t>
@@ -866,6 +875,7 @@
       </c>
     </row>
     <row r="26">
+      <c r="A26" t="inlineStr"/>
       <c r="B26" t="inlineStr">
         <is>
           <t>help.swap_card</t>
@@ -883,6 +893,7 @@
       </c>
     </row>
     <row r="27">
+      <c r="A27" t="inlineStr"/>
       <c r="B27" t="inlineStr">
         <is>
           <t>help.teleport_card</t>
@@ -900,6 +911,7 @@
       </c>
     </row>
     <row r="28">
+      <c r="A28" t="inlineStr"/>
       <c r="B28" t="inlineStr">
         <is>
           <t>help.throwing_knife</t>
@@ -917,6 +929,7 @@
       </c>
     </row>
     <row r="29">
+      <c r="A29" t="inlineStr"/>
       <c r="B29" t="inlineStr">
         <is>
           <t>help.ward_magic_card</t>
@@ -934,6 +947,7 @@
       </c>
     </row>
     <row r="30">
+      <c r="A30" t="inlineStr"/>
       <c r="B30" t="inlineStr">
         <is>
           <t>help.watchtower</t>
@@ -951,6 +965,7 @@
       </c>
     </row>
     <row r="31">
+      <c r="A31" t="inlineStr"/>
       <c r="B31" t="inlineStr">
         <is>
           <t>monster.beggar</t>
@@ -968,6 +983,7 @@
       </c>
     </row>
     <row r="32">
+      <c r="A32" t="inlineStr"/>
       <c r="B32" t="inlineStr">
         <is>
           <t>monster.big_orc</t>
@@ -985,6 +1001,7 @@
       </c>
     </row>
     <row r="33">
+      <c r="A33" t="inlineStr"/>
       <c r="B33" t="inlineStr">
         <is>
           <t>monster.big_skeleton</t>
@@ -1002,2688 +1019,2864 @@
       </c>
     </row>
     <row r="34">
+      <c r="A34" t="inlineStr"/>
       <c r="B34" t="inlineStr">
         <is>
+          <t>monster.big_skeleton_reborn</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>重组大骷髅</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>monster.big_stone</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
         <is>
           <t>大石头：左列战斗时按损失护甲伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
         <is>
           <t>monster.bone_club_skeleton</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
         <is>
           <t>骨棒骷髅</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr">
         <is>
           <t>monster.bone_courier</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>骨头快递员：每移动2次，将相邻帮助卡与战斗卡组怪物交换</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+      <c r="B38" t="inlineStr">
         <is>
           <t>monster.brainless_orc</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
         <is>
           <t>无脑兽人：战斗时本卡攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr"/>
+      <c r="B39" t="inlineStr">
         <is>
           <t>monster.dragon_cult_leader</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>龙教主：每移动3次加入龙信徒</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+      <c r="B40" t="inlineStr">
         <is>
           <t>monster.dragon_follower</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
         <is>
           <t>龙信徒：被移除时加入烈焰</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr"/>
+      <c r="B41" t="inlineStr">
         <is>
           <t>monster.executioner</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
         <is>
           <t>刽子手：每移动2次，移除九宫格上所有的龙信徒</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+      <c r="B42" t="inlineStr">
         <is>
           <t>monster.fire_bather</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
         <is>
           <t>浴火者：有烈焰时攻击+4</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+      <c r="B43" t="inlineStr">
         <is>
           <t>monster.fire_cult_leader</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
         <is>
           <t>火教主：每有一张烈焰加入战斗卡组，额外加入一张且不递归</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+      <c r="B44" t="inlineStr">
         <is>
           <t>monster.fire_dragon</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
         <is>
           <t>火龙：每移动4次移除其他普通怪物并按数量加入烈焰；烈焰帮助卡造成的伤害+1</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr"/>
+      <c r="B45" t="inlineStr">
         <is>
           <t>monster.fire_priest</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
         <is>
           <t>火焰祭司：每有一张烈焰，本卡攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+      <c r="B46" t="inlineStr">
         <is>
           <t>monster.fire_swallower</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
         <is>
           <t>吞火者：左列战斗时按损失护甲伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr"/>
+      <c r="B47" t="inlineStr">
         <is>
           <t>monster.friendly_ancient</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
         <is>
           <t>友好的远古生物：每移动3次放旋转轮</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
         <is>
           <t>monster.giant_skeleton</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
         <is>
           <t>巨大骷髅：被移除时洗入多骨虫和等级2随机怪物</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+      <c r="B49" t="inlineStr">
         <is>
           <t>monster.growing_stone</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
         <is>
           <t>增生石块：移动到左列时其他怪物获得2点护甲</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
         <is>
           <t>monster.headless_skeleton</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>无头骷髅：相邻骷髅头组合</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="B50" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
         <is>
           <t>monster.hoodlum</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
         <is>
           <t>混混：每次移动到格1时对玩家造成2点伤害</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr"/>
+      <c r="B52" t="inlineStr">
         <is>
           <t>monster.killer</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
         <is>
           <t>杀手：移动到玩家相邻格时强制战斗</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="B52" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr"/>
+      <c r="B53" t="inlineStr">
         <is>
           <t>monster.megalith</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
         <is>
           <t>巨石人：每次移动吸取相邻怪物全部护甲；累计损失10护甲洗入石人</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="B53" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr"/>
+      <c r="B54" t="inlineStr">
         <is>
           <t>monster.mist</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
         <is>
           <t>迷雾：每移动1次攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr">
         <is>
           <t>monster.multi_bone_worm</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>多骨虫：移动时与相邻两张怪物合成为巨大骷髅</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr"/>
+      <c r="B56" t="inlineStr">
         <is>
           <t>monster.observer</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
         <is>
           <t>观察者：怪物卡因怪物技能位移时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="B56" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr"/>
+      <c r="B57" t="inlineStr">
         <is>
           <t>monster.old_orc</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
         <is>
           <t>年迈兽人：战斗时恢复1且攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr"/>
+      <c r="B58" t="inlineStr">
         <is>
           <t>monster.orc_boss</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
         <is>
           <t>兽人老大：每移动2次，移除相邻格子上的怪物卡和帮助卡；依靠暴力狂移除怪物得攻击，移除帮助卡得护甲</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="B58" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr"/>
+      <c r="B59" t="inlineStr">
         <is>
           <t>monster.orc_commander</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
         <is>
           <t>兽人指挥官：每移动1次，相邻怪物攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="B59" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr"/>
+      <c r="B60" t="inlineStr">
         <is>
           <t>monster.orc_quartermaster</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
         <is>
           <t>兽人军需官：每移动2次随机强化其他怪物</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="B60" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr"/>
+      <c r="B61" t="inlineStr">
         <is>
           <t>monster.orc_warrior</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
         <is>
           <t>兽人战士：战斗时每造成2点伤害，本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="B61" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr"/>
+      <c r="B62" t="inlineStr">
         <is>
           <t>monster.pickpocket</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
         <is>
           <t>扒手：每移动3次移除相邻帮助卡</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="B62" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr"/>
+      <c r="B63" t="inlineStr">
         <is>
           <t>monster.ringleader</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
         <is>
           <t>领头人：每移动3次创建福地，怪物进入福地获得护甲和攻击；福地达到3后下一次移动造成99伤害</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="B63" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr"/>
+      <c r="B64" t="inlineStr">
         <is>
           <t>monster.rogue</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
         <is>
           <t>流氓：每损失3点护甲，相邻怪物攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="B64" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
         <is>
           <t>monster.rolling_stone_man</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
         <is>
           <t>滚石人：移动到格3时移除格6帮助卡</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
         <is>
           <t>monster.rotating_cub</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
         <is>
           <t>旋转幼崽：每移动3次旋转</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
         <is>
           <t>monster.salamander</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
         <is>
           <t>火蜥蜴：每移动3次放烈焰</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
         <is>
           <t>monster.sharp_stone</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
         <is>
           <t>尖石：护甲归零时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="B68" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
         <is>
           <t>monster.shelter_stone</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
         <is>
           <t>庇护石：其他怪物卡受到的伤害减少1点</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr"/>
+      <c r="B70" t="inlineStr">
         <is>
           <t>monster.skeleton_king</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
         <is>
           <t>骷髅王：相邻怪物被移除时获得其移除前攻击和护甲；每移动5次移除随机两张其他怪物并洗入等级2/3随机怪物</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="B70" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
         <is>
           <t>monster.skeleton_mage</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
         <is>
           <t>骷髅法师：所有怪物卡视为与本卡正交相邻</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="B71" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
         <is>
           <t>monster.skeleton_taunter</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
         <is>
           <t>骷髅嘲讽子：相邻时只能与本卡战斗</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
         <is>
           <t>monster.skull_head</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
         <is>
           <t>骷髅头：相邻无头骷髅组合</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
         <is>
           <t>monster.sky_eye</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
         <is>
           <t>空中巨眼：移动到角格时对玩家造成2点伤害</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="B74" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
         <is>
           <t>monster.smart_orc</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
         <is>
           <t>聪明兽人：每次获得攻击时，本卡额外攻击+1且不递归</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="B75" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
         <is>
           <t>monster.smuggler</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
         <is>
           <t>走私者：累计移动到玩家相邻3次时移除帮助卡并获得护甲</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="B76" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
         <is>
           <t>monster.space_master</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
         <is>
           <t>空间大师：玩家与本卡战斗后旋转一次；每移动9次从其他怪物牌组加入普通怪物</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="B77" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
         <is>
           <t>monster.stepwalker</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
         <is>
           <t>踏步行者：每移动3次与随机帮助卡交换</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="B78" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr"/>
+      <c r="B79" t="inlineStr">
         <is>
           <t>monster.stone_golem</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
         <is>
           <t>石傀儡</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="B79" t="inlineStr">
+    <row r="80">
+      <c r="A80" t="inlineStr"/>
+      <c r="B80" t="inlineStr">
         <is>
           <t>monster.stone_man</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
         <is>
           <t>石头人</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="B80" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr"/>
+      <c r="B81" t="inlineStr">
         <is>
           <t>monster.stone_shrimp</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D80" t="inlineStr">
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>石虾：玩家卡和怪物卡损失护甲时本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="B81" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr"/>
+      <c r="B82" t="inlineStr">
         <is>
           <t>monster.stone_swallower</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
         <is>
           <t>吞石者：每移动2次吸相邻怪物护甲</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="B82" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr"/>
+      <c r="B83" t="inlineStr">
         <is>
           <t>monster.stone_thrower</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
         <is>
           <t>丢石人：每移动2次消耗本卡2护甲并伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="B83" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr"/>
+      <c r="B84" t="inlineStr">
         <is>
           <t>monster.thug</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
         <is>
           <t>打手：登场在偶数边位时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="B84" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr"/>
+      <c r="B85" t="inlineStr">
         <is>
           <t>monster.vagrant</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
         <is>
           <t>流浪汉</t>
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="B85" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr"/>
+      <c r="B86" t="inlineStr">
         <is>
           <t>monster.veteran_orc</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
         <is>
           <t>历战兽人</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="B86" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr"/>
+      <c r="B87" t="inlineStr">
         <is>
           <t>monster.void_cub</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D86" t="inlineStr">
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
         <is>
           <t>虚空幼崽：每移动3次随机交换怪物</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="B87" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr"/>
+      <c r="B88" t="inlineStr">
         <is>
           <t>monster.void_lost</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
         <is>
           <t>误入虚空者</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="B88" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr"/>
+      <c r="B89" t="inlineStr">
         <is>
           <t>monster.wandering_child</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
         <is>
           <t>流浪孩童：格6攻击+2并获得先攻</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="B89" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr"/>
+      <c r="B90" t="inlineStr">
         <is>
           <t>monster.world_turning_hand</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
         <is>
           <t>转动世界的手：登场旋转一次</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="B90" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr"/>
+      <c r="B91" t="inlineStr">
         <is>
           <t>monster.young_orc</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>Monster</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Monster</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
         <is>
           <t>年轻兽人：其他怪物获得攻击时本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="B91" t="inlineStr">
+    <row r="92">
+      <c r="A92" t="inlineStr"/>
+      <c r="B92" t="inlineStr">
         <is>
           <t>deck.dragon</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>巨龙牌组</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="B92" t="inlineStr">
+    <row r="93">
+      <c r="A93" t="inlineStr"/>
+      <c r="B93" t="inlineStr">
         <is>
           <t>deck.orc_legion</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>兽人军团牌组</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="B93" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr"/>
+      <c r="B94" t="inlineStr">
         <is>
           <t>deck.skeleton_legion</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>骷髅军团牌组</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="B94" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+      <c r="B95" t="inlineStr">
         <is>
           <t>deck.stone_legion</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>石人军团牌组</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="B95" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr"/>
+      <c r="B96" t="inlineStr">
         <is>
           <t>deck.void</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>虚空牌组</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="B96" t="inlineStr">
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr">
         <is>
           <t>deck.wandering_legion</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>MonsterDeck</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D97" t="inlineStr">
         <is>
           <t>流浪军团牌组</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="B97" t="inlineStr">
+    <row r="98">
+      <c r="A98" t="inlineStr"/>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>relic.blood_shockwave</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Relic</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>血液冲击波：血量上限+4，关卡开始放入撞击教程，低血再放一张</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr">
         <is>
           <t>relic.craving</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>渴望：所有恢复血量效果翻倍</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="B98" t="inlineStr">
+    <row r="100">
+      <c r="A100" t="inlineStr"/>
+      <c r="B100" t="inlineStr">
         <is>
           <t>relic.dragon_scale_armor</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>龙鳞甲：所有怪物攻击-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="B99" t="inlineStr">
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>龙鳞甲：基础护甲+1，血量上限+6，怪物攻击-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr"/>
+      <c r="B101" t="inlineStr">
         <is>
           <t>relic.gold_armor</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>金币盔甲：金币抵消护甲伤害</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="B100" t="inlineStr">
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>金币盔甲：基础护甲+1，金币抵消护甲伤害</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr"/>
+      <c r="B102" t="inlineStr">
         <is>
           <t>relic.gold_knife</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>打金刀：击杀怪物时获得2金币</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="B101" t="inlineStr">
+    <row r="103">
+      <c r="A103" t="inlineStr"/>
+      <c r="B103" t="inlineStr">
         <is>
           <t>relic.heavy_armor</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>重盔甲：基础护甲+1，按基础护甲补当前护甲</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="B102" t="inlineStr">
+    <row r="104">
+      <c r="A104" t="inlineStr"/>
+      <c r="B104" t="inlineStr">
         <is>
           <t>relic.junk_coating</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D104" t="inlineStr">
         <is>
           <t>废物涂层：使用帮助卡时获得护甲</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="B103" t="inlineStr">
+    <row r="105">
+      <c r="A105" t="inlineStr"/>
+      <c r="B105" t="inlineStr">
         <is>
           <t>relic.junk_launcher</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D105" t="inlineStr">
         <is>
           <t>废物发射器：使用帮助卡时随机伤害</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="B104" t="inlineStr">
+    <row r="106">
+      <c r="A106" t="inlineStr"/>
+      <c r="B106" t="inlineStr">
         <is>
           <t>relic.junk_recycler</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>废物利用机：使用帮助卡时恢复2点血量</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="B105" t="inlineStr">
+    <row r="107">
+      <c r="A107" t="inlineStr"/>
+      <c r="B107" t="inlineStr">
         <is>
           <t>relic.junk_slot_machine</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>废物老虎机：使用帮助卡时随机触发九选一</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="B106" t="inlineStr">
+    <row r="108">
+      <c r="A108" t="inlineStr"/>
+      <c r="B108" t="inlineStr">
         <is>
           <t>relic.lucky_coin</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D108" t="inlineStr">
         <is>
           <t>幸运硬币：击杀精英/层主时加入金币卡</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="B107" t="inlineStr">
+    <row r="109">
+      <c r="A109" t="inlineStr"/>
+      <c r="B109" t="inlineStr">
         <is>
           <t>relic.phoenix_feather</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>凤凰羽毛：致命伤害免死</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="B108" t="inlineStr">
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>凤凰羽毛：血量上限+8，致命伤害免死</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr"/>
+      <c r="B110" t="inlineStr">
         <is>
           <t>relic.potion_bag</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>药水袋：每关卡开始加入两张恢复药水</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="B109" t="inlineStr">
+    <row r="111">
+      <c r="A111" t="inlineStr"/>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>relic.rotation_button</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Relic</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>旋转按钮：每关卡开始放入旋转轮</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr"/>
+      <c r="B112" t="inlineStr">
         <is>
           <t>relic.shield_knife</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>打盾刀：击杀怪物时获得护甲</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="B110" t="inlineStr">
+    <row r="113">
+      <c r="A113" t="inlineStr"/>
+      <c r="B113" t="inlineStr">
         <is>
           <t>relic.sling</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>弹弓：击杀怪物时随机伤害</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="B111" t="inlineStr">
+    <row r="114">
+      <c r="A114" t="inlineStr"/>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>relic.swap_button</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Relic</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>交换按钮：每关卡开始放入交换卡</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr"/>
+      <c r="B115" t="inlineStr">
         <is>
           <t>relic.throwing_knife_bag</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>飞刀袋：每关卡开始加入两张飞刀</t>
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="B112" t="inlineStr">
+    <row r="116">
+      <c r="A116" t="inlineStr"/>
+      <c r="B116" t="inlineStr">
         <is>
           <t>relic.vitality_amulet</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D116" t="inlineStr">
         <is>
           <t>活力护符：血量上限+6，关卡结束恢复6</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="B113" t="inlineStr">
+    <row r="117">
+      <c r="A117" t="inlineStr"/>
+      <c r="B117" t="inlineStr">
         <is>
           <t>relic.wood_armor</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C117" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D117" t="inlineStr">
         <is>
           <t>木甲：血量上限+2，木套装额外+8</t>
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="B114" t="inlineStr">
+    <row r="118">
+      <c r="A118" t="inlineStr"/>
+      <c r="B118" t="inlineStr">
         <is>
           <t>relic.wood_shield</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C118" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D118" t="inlineStr">
         <is>
           <t>木盾：基础护甲+1，木套装额外+2</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="B115" t="inlineStr">
+    <row r="119">
+      <c r="A119" t="inlineStr"/>
+      <c r="B119" t="inlineStr">
         <is>
           <t>relic.wood_sword</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>Relic</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D119" t="inlineStr">
         <is>
           <t>木剑：攻击+1，木套装额外+2</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="B116" t="inlineStr">
+    <row r="120">
+      <c r="A120" t="inlineStr"/>
+      <c r="B120" t="inlineStr">
         <is>
           <t>Fountain</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C120" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr">
+      <c r="D120" t="inlineStr">
         <is>
           <t>温泉房</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="B117" t="inlineStr">
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="inlineStr">
         <is>
           <t>Gold</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C121" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D121" t="inlineStr">
         <is>
           <t>金币房</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="B118" t="inlineStr">
+    <row r="122">
+      <c r="A122" t="inlineStr"/>
+      <c r="B122" t="inlineStr">
         <is>
           <t>Shop</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C122" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D122" t="inlineStr">
         <is>
           <t>商店</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="B119" t="inlineStr">
+    <row r="123">
+      <c r="A123" t="inlineStr"/>
+      <c r="B123" t="inlineStr">
         <is>
           <t>Tavern</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
+      <c r="C123" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="D119" t="inlineStr">
+      <c r="D123" t="inlineStr">
         <is>
           <t>酒馆</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="B120" t="inlineStr">
+    <row r="124">
+      <c r="A124" t="inlineStr"/>
+      <c r="B124" t="inlineStr">
         <is>
           <t>Treasure</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D124" t="inlineStr">
         <is>
           <t>宝箱房</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="B121" t="inlineStr">
+    <row r="125">
+      <c r="A125" t="inlineStr"/>
+      <c r="B125" t="inlineStr">
         <is>
           <t>skill.absorb_bone</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
         <is>
           <t>吸骨：相邻怪物被移除时获得其移除前攻击和护甲</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="B122" t="inlineStr">
+    <row r="126">
+      <c r="A126" t="inlineStr"/>
+      <c r="B126" t="inlineStr">
         <is>
           <t>skill.absorb_stone</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
         <is>
           <t>吸石：每次移动吸取相邻怪物全部护甲</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="B123" t="inlineStr">
+    <row r="127">
+      <c r="A127" t="inlineStr"/>
+      <c r="B127" t="inlineStr">
         <is>
           <t>skill.air_strike</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
         <is>
           <t>空中打击：移动到角格时对玩家造成2点伤害</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="B124" t="inlineStr">
+    <row r="128">
+      <c r="A128" t="inlineStr"/>
+      <c r="B128" t="inlineStr">
         <is>
           <t>skill.arsenal</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D124" t="inlineStr">
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
         <is>
           <t>军械库：关卡结束加入飞刀/爆弹/破击锤之一</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="B125" t="inlineStr">
+    <row r="129">
+      <c r="A129" t="inlineStr"/>
+      <c r="B129" t="inlineStr">
         <is>
           <t>skill.battle_hardened</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
         <is>
           <t>历战：战斗时攻击+2，换敌复原</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="B126" t="inlineStr">
+    <row r="130">
+      <c r="A130" t="inlineStr"/>
+      <c r="B130" t="inlineStr">
         <is>
           <t>skill.beggar_bond</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
         <is>
           <t>丐帮同心：每移动5次洗入乞丐</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="B127" t="inlineStr">
+    <row r="131">
+      <c r="A131" t="inlineStr"/>
+      <c r="B131" t="inlineStr">
         <is>
           <t>skill.blessing</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
         <is>
           <t>庇佑：下一次受到伤害时，该次伤害变为0</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="B128" t="inlineStr">
+    <row r="132">
+      <c r="A132" t="inlineStr"/>
+      <c r="B132" t="inlineStr">
         <is>
           <t>skill.bloodthirst</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
         <is>
           <t>嗜血：战斗时每造成2点伤害，本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="B129" t="inlineStr">
+    <row r="133">
+      <c r="A133" t="inlineStr"/>
+      <c r="B133" t="inlineStr">
         <is>
           <t>skill.breathe_fire</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
         <is>
           <t>喷火：每移动3次放烈焰</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="B130" t="inlineStr">
+    <row r="134">
+      <c r="A134" t="inlineStr"/>
+      <c r="B134" t="inlineStr">
         <is>
           <t>skill.call_followers</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
         <is>
           <t>呼唤信徒：每移动3次加入龙信徒</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="B131" t="inlineStr">
+    <row r="135">
+      <c r="A135" t="inlineStr"/>
+      <c r="B135" t="inlineStr">
         <is>
           <t>skill.delivery</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
         <is>
           <t>快递：每移动2次，将相邻帮助卡与战斗卡组怪物交换</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="B132" t="inlineStr">
+    <row r="136">
+      <c r="A136" t="inlineStr"/>
+      <c r="B136" t="inlineStr">
         <is>
           <t>skill.devotion</t>
         </is>
       </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
         <is>
           <t>献身：被移除时加入烈焰</t>
         </is>
       </c>
     </row>
-    <row r="133">
-      <c r="B133" t="inlineStr">
+    <row r="137">
+      <c r="A137" t="inlineStr"/>
+      <c r="B137" t="inlineStr">
         <is>
           <t>skill.easy_road</t>
         </is>
       </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
         <is>
           <t>轻车熟路：关卡结束白色帮助卡三选一</t>
         </is>
       </c>
     </row>
-    <row r="134">
-      <c r="B134" t="inlineStr">
+    <row r="138">
+      <c r="A138" t="inlineStr"/>
+      <c r="B138" t="inlineStr">
         <is>
           <t>skill.even_hatred</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
         <is>
           <t>偶数仇恨：对偶数等级怪物造成双倍伤害</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="B135" t="inlineStr">
+    <row r="139">
+      <c r="A139" t="inlineStr"/>
+      <c r="B139" t="inlineStr">
         <is>
           <t>skill.fall_apart</t>
         </is>
       </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
         <is>
           <t>散架：被移除时洗入骷髅头与无头骷髅</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="B136" t="inlineStr">
+    <row r="140">
+      <c r="A140" t="inlineStr"/>
+      <c r="B140" t="inlineStr">
         <is>
           <t>skill.falling_rocks</t>
         </is>
       </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
         <is>
           <t>落石：累计损失10护甲洗入石人</t>
         </is>
       </c>
     </row>
-    <row r="137">
-      <c r="B137" t="inlineStr">
+    <row r="141">
+      <c r="A141" t="inlineStr"/>
+      <c r="B141" t="inlineStr">
         <is>
           <t>skill.fight_me</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
         <is>
           <t>和我打！：相邻玩家与其他怪物战斗时改为与本卡战斗</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="B138" t="inlineStr">
+    <row r="142">
+      <c r="A142" t="inlineStr"/>
+      <c r="B142" t="inlineStr">
         <is>
           <t>skill.find_weakness</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
         <is>
           <t>发现弱点：福地达到3后下一次移动造成99伤害</t>
         </is>
       </c>
     </row>
-    <row r="139">
-      <c r="B139" t="inlineStr">
+    <row r="143">
+      <c r="A143" t="inlineStr"/>
+      <c r="B143" t="inlineStr">
         <is>
           <t>skill.fire_power</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
         <is>
           <t>火之力：每有一张烈焰，本卡攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="140">
-      <c r="B140" t="inlineStr">
+    <row r="144">
+      <c r="A144" t="inlineStr"/>
+      <c r="B144" t="inlineStr">
         <is>
           <t>skill.first_strike</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
         <is>
           <t>先攻：持有先攻技能</t>
         </is>
       </c>
     </row>
-    <row r="141">
-      <c r="B141" t="inlineStr">
+    <row r="145">
+      <c r="A145" t="inlineStr"/>
+      <c r="B145" t="inlineStr">
         <is>
           <t>skill.flame_boiling</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
         <is>
           <t>烈焰沸腾：烈焰帮助卡造成的伤害+1</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="B142" t="inlineStr">
+    <row r="146">
+      <c r="A146" t="inlineStr"/>
+      <c r="B146" t="inlineStr">
         <is>
           <t>skill.flame_breath</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
         <is>
           <t>烈焰吐息：每移动4次移除其他普通怪物并按数量加入烈焰</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="B143" t="inlineStr">
+    <row r="147">
+      <c r="A147" t="inlineStr"/>
+      <c r="B147" t="inlineStr">
         <is>
           <t>skill.fracture_fall_apart</t>
         </is>
       </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
         <is>
           <t>折损散架：被移除时洗入多骨虫和等级2随机怪物</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="B144" t="inlineStr">
+    <row r="148">
+      <c r="A148" t="inlineStr"/>
+      <c r="B148" t="inlineStr">
         <is>
           <t>skill.gear_delivery</t>
         </is>
       </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
         <is>
           <t>发装备了！：每移动2次随机强化其他怪物</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="B145" t="inlineStr">
+    <row r="149">
+      <c r="A149" t="inlineStr"/>
+      <c r="B149" t="inlineStr">
         <is>
           <t>skill.gift</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
         <is>
           <t>礼物：每移动3次放旋转轮</t>
         </is>
       </c>
     </row>
-    <row r="146">
-      <c r="B146" t="inlineStr">
+    <row r="150">
+      <c r="A150" t="inlineStr"/>
+      <c r="B150" t="inlineStr">
         <is>
           <t>skill.give_punch</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
         <is>
           <t>给你一拳：登场在偶数边位时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="147">
-      <c r="B147" t="inlineStr">
+    <row r="151">
+      <c r="A151" t="inlineStr"/>
+      <c r="B151" t="inlineStr">
         <is>
           <t>skill.guide</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
         <is>
           <t>引路：每移动3次创建福地，怪物进入福地获得护甲和攻击</t>
         </is>
       </c>
     </row>
-    <row r="148">
-      <c r="B148" t="inlineStr">
+    <row r="152">
+      <c r="A152" t="inlineStr"/>
+      <c r="B152" t="inlineStr">
         <is>
           <t>skill.hard</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
         <is>
           <t>坚硬：左列战斗时按损失护甲伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="149">
-      <c r="B149" t="inlineStr">
+    <row r="153">
+      <c r="A153" t="inlineStr"/>
+      <c r="B153" t="inlineStr">
         <is>
           <t>skill.hard_skin</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
         <is>
           <t>硬皮：血量上限+10，关卡结束恢复10</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="B150" t="inlineStr">
+    <row r="154">
+      <c r="A154" t="inlineStr"/>
+      <c r="B154" t="inlineStr">
         <is>
           <t>skill.hoodlum</t>
         </is>
       </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
         <is>
           <t>混的人：每次移动到格1时对玩家造成2点伤害</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="B151" t="inlineStr">
+    <row r="155">
+      <c r="A155" t="inlineStr"/>
+      <c r="B155" t="inlineStr">
         <is>
           <t>skill.hot_observation</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
         <is>
           <t>灼热观察：怪物卡因怪物技能位移时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="B152" t="inlineStr">
+    <row r="156">
+      <c r="A156" t="inlineStr"/>
+      <c r="B156" t="inlineStr">
         <is>
           <t>skill.intense_burning</t>
         </is>
       </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
         <is>
           <t>剧烈燃烧：每有一张烈焰加入战斗卡组，额外加入一张且不递归</t>
         </is>
       </c>
     </row>
-    <row r="153">
-      <c r="B153" t="inlineStr">
+    <row r="157">
+      <c r="A157" t="inlineStr"/>
+      <c r="B157" t="inlineStr">
         <is>
           <t>skill.learning_growth</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
         <is>
           <t>学习成长：其他怪物获得攻击时本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="B154" t="inlineStr">
+    <row r="158">
+      <c r="A158" t="inlineStr"/>
+      <c r="B158" t="inlineStr">
         <is>
           <t>skill.love_fire</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
         <is>
           <t>恋火：有烈焰时攻击+4</t>
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="B155" t="inlineStr">
+    <row r="159">
+      <c r="A159" t="inlineStr"/>
+      <c r="B159" t="inlineStr">
         <is>
           <t>skill.mixed_bones</t>
         </is>
       </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
         <is>
           <t>混合骨头：每移动5次移除随机两张其他怪物并洗入等级2/3随机怪物</t>
         </is>
       </c>
     </row>
-    <row r="156">
-      <c r="B156" t="inlineStr">
+    <row r="160">
+      <c r="A160" t="inlineStr"/>
+      <c r="B160" t="inlineStr">
         <is>
           <t>skill.monster_battle_hardened</t>
         </is>
       </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
         <is>
           <t>历战怪物：战斗时本卡攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="B157" t="inlineStr">
+    <row r="161">
+      <c r="A161" t="inlineStr"/>
+      <c r="B161" t="inlineStr">
         <is>
           <t>skill.orc_tactics</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
         <is>
           <t>兽人战术：每移动1次，相邻怪物攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="158">
-      <c r="B158" t="inlineStr">
+    <row r="162">
+      <c r="A162" t="inlineStr"/>
+      <c r="B162" t="inlineStr">
         <is>
           <t>skill.otherworld_help</t>
         </is>
       </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
         <is>
           <t>异界帮助：每移动9次从其他怪物牌组加入普通怪物</t>
         </is>
       </c>
     </row>
-    <row r="159">
-      <c r="B159" t="inlineStr">
+    <row r="163">
+      <c r="A163" t="inlineStr"/>
+      <c r="B163" t="inlineStr">
         <is>
           <t>skill.random_walk</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
         <is>
           <t>乱步：每移动3次与随机帮助卡交换</t>
         </is>
       </c>
     </row>
-    <row r="160">
-      <c r="B160" t="inlineStr">
+    <row r="164">
+      <c r="A164" t="inlineStr"/>
+      <c r="B164" t="inlineStr">
         <is>
           <t>skill.range_expand</t>
         </is>
       </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
         <is>
           <t>范围扩大：所有怪物卡视为与本卡正交相邻</t>
         </is>
       </c>
     </row>
-    <row r="161">
-      <c r="B161" t="inlineStr">
+    <row r="165">
+      <c r="A165" t="inlineStr"/>
+      <c r="B165" t="inlineStr">
         <is>
           <t>skill.rascality</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
         <is>
           <t>痞气：每损失3点护甲，相邻怪物攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="162">
-      <c r="B162" t="inlineStr">
+    <row r="166">
+      <c r="A166" t="inlineStr"/>
+      <c r="B166" t="inlineStr">
         <is>
           <t>skill.recombine_body</t>
         </is>
       </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
         <is>
           <t>重新组合身：相邻无头骷髅组合</t>
         </is>
       </c>
     </row>
-    <row r="163">
-      <c r="B163" t="inlineStr">
+    <row r="167">
+      <c r="A167" t="inlineStr"/>
+      <c r="B167" t="inlineStr">
         <is>
           <t>skill.recombine_head</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
         <is>
           <t>重新组合头：相邻骷髅头组合</t>
         </is>
       </c>
     </row>
-    <row r="164">
-      <c r="B164" t="inlineStr">
+    <row r="168">
+      <c r="A168" t="inlineStr"/>
+      <c r="B168" t="inlineStr">
         <is>
           <t>skill.relentless_chase</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
         <is>
           <t>不休追击：移动到玩家相邻格时强制战斗</t>
         </is>
       </c>
     </row>
-    <row r="165">
-      <c r="B165" t="inlineStr">
+    <row r="169">
+      <c r="A169" t="inlineStr"/>
+      <c r="B169" t="inlineStr">
         <is>
           <t>skill.rolling_crush</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
         <is>
           <t>滚动碾压：移动到格3时移除格6帮助卡</t>
         </is>
       </c>
     </row>
-    <row r="166">
-      <c r="B166" t="inlineStr">
+    <row r="170">
+      <c r="A170" t="inlineStr"/>
+      <c r="B170" t="inlineStr">
         <is>
           <t>skill.rotate_lover</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
         <is>
           <t>爱好旋转：每移动3次旋转</t>
         </is>
       </c>
     </row>
-    <row r="167">
-      <c r="B167" t="inlineStr">
+    <row r="171">
+      <c r="A171" t="inlineStr"/>
+      <c r="B171" t="inlineStr">
         <is>
           <t>skill.sacrifice</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
         <is>
           <t>献祭：每移动2次，移除九宫格上所有的龙信徒</t>
         </is>
       </c>
     </row>
-    <row r="168">
-      <c r="B168" t="inlineStr">
+    <row r="172">
+      <c r="A172" t="inlineStr"/>
+      <c r="B172" t="inlineStr">
         <is>
           <t>skill.sharp_stone</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
         <is>
           <t>尖石：护甲归零时伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="169">
-      <c r="B169" t="inlineStr">
+    <row r="173">
+      <c r="A173" t="inlineStr"/>
+      <c r="B173" t="inlineStr">
         <is>
           <t>skill.smart</t>
         </is>
       </c>
-      <c r="C169" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D169" t="inlineStr">
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
         <is>
           <t>大聪明：每次获得攻击时，本卡额外攻击+1且不递归</t>
         </is>
       </c>
     </row>
-    <row r="170">
-      <c r="B170" t="inlineStr">
+    <row r="174">
+      <c r="A174" t="inlineStr"/>
+      <c r="B174" t="inlineStr">
         <is>
           <t>skill.space_mastery</t>
         </is>
       </c>
-      <c r="C170" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D170" t="inlineStr">
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
         <is>
           <t>空间掌握：玩家与本卡战斗后旋转一次</t>
         </is>
       </c>
     </row>
-    <row r="171">
-      <c r="B171" t="inlineStr">
+    <row r="175">
+      <c r="A175" t="inlineStr"/>
+      <c r="B175" t="inlineStr">
         <is>
           <t>skill.stocking</t>
         </is>
       </c>
-      <c r="C171" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D171" t="inlineStr">
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
         <is>
           <t>进货：累计移动到玩家相邻3次时移除帮助卡并获得护甲</t>
         </is>
       </c>
     </row>
-    <row r="172">
-      <c r="B172" t="inlineStr">
+    <row r="176">
+      <c r="A176" t="inlineStr"/>
+      <c r="B176" t="inlineStr">
         <is>
           <t>skill.stone_growth</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D172" t="inlineStr">
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
         <is>
           <t>石增长：移动到左列时其他怪物获得2点护甲</t>
         </is>
       </c>
     </row>
-    <row r="173">
-      <c r="B173" t="inlineStr">
+    <row r="177">
+      <c r="A177" t="inlineStr"/>
+      <c r="B177" t="inlineStr">
         <is>
           <t>skill.stone_lover</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D173" t="inlineStr">
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
         <is>
           <t>石头爱好者：玩家卡和怪物卡损失护甲时本卡攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="174">
-      <c r="B174" t="inlineStr">
+    <row r="178">
+      <c r="A178" t="inlineStr"/>
+      <c r="B178" t="inlineStr">
         <is>
           <t>skill.stone_shelter</t>
         </is>
       </c>
-      <c r="C174" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D174" t="inlineStr">
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
         <is>
           <t>石庇护：其他怪物卡受到的伤害减少1点</t>
         </is>
       </c>
     </row>
-    <row r="175">
-      <c r="B175" t="inlineStr">
+    <row r="179">
+      <c r="A179" t="inlineStr"/>
+      <c r="B179" t="inlineStr">
         <is>
           <t>skill.stray_cub</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D175" t="inlineStr">
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
         <is>
           <t>流浪幼崽：格6攻击+2并获得先攻</t>
         </is>
       </c>
     </row>
-    <row r="176">
-      <c r="B176" t="inlineStr">
+    <row r="180">
+      <c r="A180" t="inlineStr"/>
+      <c r="B180" t="inlineStr">
         <is>
           <t>skill.stroll</t>
         </is>
       </c>
-      <c r="C176" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr">
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
         <is>
           <t>漫步：每移动1次攻击+2</t>
         </is>
       </c>
     </row>
-    <row r="177">
-      <c r="B177" t="inlineStr">
+    <row r="181">
+      <c r="A181" t="inlineStr"/>
+      <c r="B181" t="inlineStr">
         <is>
           <t>skill.strong_combo</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
         <is>
           <t>强力组合：移动时与相邻两张怪物合成为巨大骷髅</t>
         </is>
       </c>
     </row>
-    <row r="178">
-      <c r="B178" t="inlineStr">
+    <row r="182">
+      <c r="A182" t="inlineStr"/>
+      <c r="B182" t="inlineStr">
         <is>
           <t>skill.survival_wisdom</t>
         </is>
       </c>
-      <c r="C178" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D178" t="inlineStr">
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
         <is>
           <t>生存智慧：战斗时恢复1且攻击+1</t>
         </is>
       </c>
     </row>
-    <row r="179">
-      <c r="B179" t="inlineStr">
+    <row r="183">
+      <c r="A183" t="inlineStr"/>
+      <c r="B183" t="inlineStr">
         <is>
           <t>skill.swallow_stone</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D179" t="inlineStr">
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
         <is>
           <t>吞石：每移动2次吸相邻怪物护甲</t>
         </is>
       </c>
     </row>
-    <row r="180">
-      <c r="B180" t="inlineStr">
+    <row r="184">
+      <c r="A184" t="inlineStr"/>
+      <c r="B184" t="inlineStr">
         <is>
           <t>skill.taunt</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
         <is>
           <t>嘲讽：相邻时只能与本卡战斗</t>
         </is>
       </c>
     </row>
-    <row r="181">
-      <c r="B181" t="inlineStr">
+    <row r="185">
+      <c r="A185" t="inlineStr"/>
+      <c r="B185" t="inlineStr">
         <is>
           <t>skill.thief_claims</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D181" t="inlineStr">
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
         <is>
           <t>东西归我了！：每移动3次移除相邻帮助卡</t>
         </is>
       </c>
     </row>
-    <row r="182">
-      <c r="B182" t="inlineStr">
+    <row r="186">
+      <c r="A186" t="inlineStr"/>
+      <c r="B186" t="inlineStr">
         <is>
           <t>skill.thorn_skin</t>
         </is>
       </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D182" t="inlineStr">
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
         <is>
           <t>刺皮：战斗时对怪物造成等同其攻击的伤害</t>
         </is>
       </c>
     </row>
-    <row r="183">
-      <c r="B183" t="inlineStr">
+    <row r="187">
+      <c r="A187" t="inlineStr"/>
+      <c r="B187" t="inlineStr">
         <is>
           <t>skill.throw_stone</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D183" t="inlineStr">
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
         <is>
           <t>丢石头：每移动2次消耗本卡2护甲并伤害玩家</t>
         </is>
       </c>
     </row>
-    <row r="184">
-      <c r="B184" t="inlineStr">
+    <row r="188">
+      <c r="A188" t="inlineStr"/>
+      <c r="B188" t="inlineStr">
         <is>
           <t>skill.tower_child</t>
         </is>
       </c>
-      <c r="C184" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D184" t="inlineStr">
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
         <is>
           <t>塔之子：关卡开始放入倍增塔</t>
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="B185" t="inlineStr">
+    <row r="189">
+      <c r="A189" t="inlineStr"/>
+      <c r="B189" t="inlineStr">
         <is>
           <t>skill.turn_world</t>
         </is>
       </c>
-      <c r="C185" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D185" t="inlineStr">
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
         <is>
           <t>转动：登场旋转一次</t>
         </is>
       </c>
     </row>
-    <row r="186">
-      <c r="B186" t="inlineStr">
+    <row r="190">
+      <c r="A190" t="inlineStr"/>
+      <c r="B190" t="inlineStr">
         <is>
           <t>skill.unstable</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D186" t="inlineStr">
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
         <is>
           <t>不稳定：每移动3次随机交换怪物</t>
         </is>
       </c>
     </row>
-    <row r="187">
-      <c r="B187" t="inlineStr">
+    <row r="191">
+      <c r="A191" t="inlineStr"/>
+      <c r="B191" t="inlineStr">
         <is>
           <t>skill.violence_maniac</t>
         </is>
       </c>
-      <c r="C187" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D187" t="inlineStr">
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
         <is>
           <t>暴力狂：每移动2次，移除相邻格子上的怪物卡和帮助卡</t>
         </is>
       </c>
     </row>
-    <row r="188">
-      <c r="B188" t="inlineStr">
+    <row r="192">
+      <c r="A192" t="inlineStr"/>
+      <c r="B192" t="inlineStr">
         <is>
           <t>skill.violence_nutrition</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
-        <is>
-          <t>Skill</t>
-        </is>
-      </c>
-      <c r="D188" t="inlineStr">
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Skill</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
         <is>
           <t>暴力即养分：依靠暴力狂移除怪物得攻击，移除帮助卡得护甲</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>Attack</t>
-        </is>
-      </c>
-      <c r="C189" t="inlineStr">
-        <is>
-          <t>ChoiceOption</t>
-        </is>
-      </c>
-      <c r="D189" t="inlineStr">
-        <is>
-          <t>攻击+1</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>Armor</t>
-        </is>
-      </c>
-      <c r="C190" t="inlineStr">
-        <is>
-          <t>ChoiceOption</t>
-        </is>
-      </c>
-      <c r="D190" t="inlineStr">
-        <is>
-          <t>护甲+1</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>Hp</t>
-        </is>
-      </c>
-      <c r="C191" t="inlineStr">
-        <is>
-          <t>ChoiceOption</t>
-        </is>
-      </c>
-      <c r="D191" t="inlineStr">
-        <is>
-          <t>血量上限与当前血量+2</t>
         </is>
       </c>
     </row>

</xml_diff>